<commit_message>
fix(policy): sync bundled filter lists to the registry-derived engine list (27 -> 80 packages)
The desktop xlsx was registry-synced on 2026-06-26 but never committed, and
the web bundled CSV was a stale 27-package snapshot of the old policy. The
two files are read by the SAME parity harness (desktop side reads the xlsx,
web side reads the CSV), so the drift was a latent parity break, and it made
the audio/navigation class look arbitrary: Spotify was filtered but YouTube
Music, Maps, iHeartRadio Family, Pandora, and Audible were not.

Both files now carry the identical 80-package registry-derived policy,
including the full audio/navigation class, and the typo'd com.anroid.launcher3
entry is gone. The filter-vs-background overlap is now {Spotify, Maps} — both
declared by the config notice whenever both features are enabled.
</commit_message>
<xml_diff>
--- a/apps_to_filter_files/Chronicle_Android_raw_data_preprocessor_apps_to_filter.xlsx
+++ b/apps_to_filter_files/Chronicle_Android_raw_data_preprocessor_apps_to_filter.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,26 +413,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>app_package_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>known_application_labels</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>app_filter_category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>filter_bool</t>
         </is>
@@ -453,17 +441,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>com.sec.android.app.clockpackage</t>
+          <t>android</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clock, Reloj</t>
+          <t>Android System, Sistema Android, System</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -473,17 +461,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>com.android.deskclock</t>
+          <t>com.amazon.csapp</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clock, Reloj</t>
+          <t>Help</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -493,17 +481,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>com.android.cellbroadcastreceiver</t>
+          <t>com.amazon.firelauncher</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wireless emergency alerts, Wireless Emergency Alerts, com.android.cellbroadcastreceiver</t>
+          <t>Amazon Fire Launcher, Home Pages</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -513,17 +501,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>android</t>
+          <t>com.amazon.parentalcontrols</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>System, Android System, Sistema Android</t>
+          <t>Profile and parental controls</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Android System</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -533,17 +521,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>com.wssyncmldm</t>
+          <t>com.amazon.settings</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Software update, Actualización de software</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -553,17 +541,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>com.samsung.android.samsungpassautofill</t>
+          <t>com.amazon.settings.systemupdates</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Autofill with Samsung Pass, Autorrellenar (Samsung Pass)</t>
+          <t>System Updates</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -573,17 +561,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>com.samsung.android.samsungpass</t>
+          <t>com.amazon.smartgenie</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Samsung Pass</t>
+          <t>Device Dashboard</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -593,17 +581,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>com.osp.app.signin</t>
+          <t>com.amazon.ssmsys</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Samsung account</t>
+          <t>System Status Monitor</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -613,17 +601,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>com.google.android.packageinstaller</t>
+          <t>com.android.calculator2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Package installer, Instalador de paquetes</t>
+          <t>Calculator</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -633,17 +621,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>com.verizon.mips.services</t>
+          <t>com.android.cellbroadcastreceiver</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>My Verizon Services</t>
+          <t>Wireless Emergency Alerts, Wireless emergency alerts, com.android.cellbroadcastreceiver</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -653,17 +641,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>com.google.android.permissioncontroller</t>
+          <t>com.android.deskclock</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Permission controller, Controlador de permisos</t>
+          <t>Clock, Reloj</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -673,17 +661,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>com.google.android.gms</t>
+          <t>com.android.documentsui</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Google Play services, Servicios de Google Play</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -693,17 +681,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>com.android.systemui</t>
+          <t>com.android.intentresolver</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>System, System UI, UI sistema, IU del sistema, Keyguard</t>
+          <t>IntentResolver</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -713,17 +701,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>com.android.server.telecom</t>
+          <t>com.android.launcher3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Phone Calls, Phone calls, Llamadas telef�nicas, Llamadas telefonicas, Llamadas telefónicas, Call Management, Call management, Phone</t>
+          <t>Launcher3, Quickstep</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -733,17 +721,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>com.google.android.dialer</t>
+          <t>com.android.printspooler</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Print Spooler</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -753,17 +741,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>com.samsung.android.incallui</t>
+          <t>com.android.providers.downloads.ui</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Call, Llamar</t>
+          <t>Downloads</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -773,17 +761,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>com.spotify.music</t>
+          <t>com.android.settings</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>Ajustes, Configuración, Settings</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Audio</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -793,17 +781,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>com.openlattice.chronicle</t>
+          <t>com.android.settings.intelligence</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>chronicle</t>
+          <t>Settings Suggestions, Settings suggestions, Sugerencias de ajustes</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Chronicle</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -813,17 +801,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>com.amazon.firelauncher</t>
+          <t>com.android.systemui</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Home Pages, Amazon Fire Launcher</t>
+          <t>IU del sistema, Keyguard, System, System UI, UI sistema</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -833,17 +821,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>com.sec.android.app.launcher</t>
+          <t>com.applovin.array.apphub.tmobile</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>One UI Home, Inicio de One UI</t>
+          <t>AppHub</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -853,17 +841,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>com.motorola.launcher3</t>
+          <t>com.att.myWireless</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Moto App Launcher</t>
+          <t>myAT&amp;T</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -873,17 +861,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>com.google.android.apps.nexuslauncher</t>
+          <t>com.audible.application.kindle</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pixel Launcher</t>
+          <t>Audible</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>audio</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -893,17 +881,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>com.android.launcher3</t>
+          <t>com.aura.news.hashtag.news</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Quickstep, Launcher3</t>
+          <t>#news</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>lockscreen-phantom</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -913,17 +901,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>com.lge.launcher3</t>
+          <t>com.byteapps.rokuremote.beta</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>RoByte</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>external-remote</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -933,17 +921,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>com.android.settings</t>
+          <t>com.clearchannel.iheartkids.freetime</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Settings, Ajustes, Configuración</t>
+          <t>iHeartRadio Family</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>audio</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -953,17 +941,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>com.android.settings.intelligence</t>
+          <t>com.dti.att</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Settings Suggestions, Settings suggestions, Sugerencias de ajustes</t>
+          <t>Mobile Services Manager</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -973,17 +961,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>com.samsung.android.app.telephonyui</t>
+          <t>com.example.screentime</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Call settings, Ajustes de llamada</t>
+          <t>ScreenTime</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -993,17 +981,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>com.tcl.android.launcher</t>
+          <t>com.google.android.apps.maps</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Launcher</t>
+          <t>Maps</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>navigation</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1013,17 +1001,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>com.mediatek.batterywarning</t>
+          <t>com.google.android.apps.nbu.files</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>com.mediatek.batterywarning</t>
+          <t>Files by Google</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Background Process</t>
+          <t>system</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1033,17 +1021,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>jp.kyocera.kyocerahome.launcher</t>
+          <t>com.google.android.apps.youtube.music</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Standard Home</t>
+          <t>YouTube Music</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Home Screen</t>
+          <t>audio</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1053,20 +1041,1000 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>com.google.android.captiveportallogin</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Captive Portal Login</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>com.google.android.cellbroadcastreceiver</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Wireless Emergency Alerts</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>com.google.android.contacts</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>com.google.android.deskclock</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Clock</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>com.google.android.dialer</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>com.google.android.gm</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Gmail</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>non-child-productivity</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>com.google.android.gm.lite</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Gmail</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>non-child-productivity</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>com.google.android.gms</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Google Play services, Servicios de Google Play</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>com.google.android.gms.supervision</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>System parental controls</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>com.google.android.packageinstaller</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Instalador de paquetes, Package installer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>com.google.android.permissioncontroller</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Controlador de permisos, Permission controller</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>com.lge.launcher3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>com.manageengine.mdm.android</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ManageEngine MDM</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>com.mediatek.batterywarning</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>com.mediatek.batterywarning</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>com.mediatek.duraspeed</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DuraSpeed</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>com.metro.minus1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Metro Play</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>carrier</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>com.metropcs.metrozone</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>metroZone</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>carrier</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>com.microsoft.office.excel</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>non-child-productivity</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>com.microsoft.skydrive</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>OneDrive</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>non-child-productivity</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>com.motorola.launcher3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Moto App Launcher</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>com.openlattice.chronicle</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>chronicle</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>com.pandora.android</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Pandora</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>audio</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>com.pls247.mobile.pls_android</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PLS Mobile</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>carrier</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>com.qlixar.qlixar</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Qlixar News</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>lockscreen-phantom</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>com.samsung.android.app.contacts</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Contacts</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>com.samsung.android.app.dressroom</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Wallpaper and style</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>com.samsung.android.app.routines</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Modes and Routines</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>com.samsung.android.bixby.agent</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bixby Voice</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>com.samsung.android.dialer</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>com.samsung.android.forest</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Digital Wellbeing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>com.samsung.android.incallui</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Call, Llamar</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>com.sec.android.app.clockpackage</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Clock, Reloj</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>com.sec.android.app.launcher</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Inicio de One UI, One UI Home</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>com.sec.android.daemonapp</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>com.spotify.music</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>audio</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>com.squareup.cash</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Cash App</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>non-child-productivity</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>com.tcl.android.launcher</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Launcher</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>com.wefi.qlink</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Free Wi-Fi</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>com.wssyncmldm</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Actualización de software, Software update</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>com.zhiliao.musically.livewallpaper</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>TickTock Video Wallpaper by TikTok</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>jp.kyocera.kyocerahome.launcher</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Standard Home</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>my.photo.picture.keyboard.app.keyboard.theme</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>#Love Keyboard</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>com.android.server.telecom</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Phone Calls, Phone calls, Llamadas telef�nicas, Llamadas telefonicas, Llamadas telefónicas, Call Management, Call management, Phone</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>com.google.android.apps.nexuslauncher</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Pixel Launcher</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>com.k2.consolelauncher</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>Console Launcher</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Home Screen</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>com.osp.app.signin</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Samsung account</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>com.samsung.android.app.telephonyui</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Call settings, Ajustes de llamada</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>com.samsung.android.samsungpass</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Samsung Pass</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>com.samsung.android.samsungpassautofill</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Autofill with Samsung Pass, Autorrellenar (Samsung Pass)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>com.verizon.mips.services</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>My Verizon Services</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>system-defensive</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>